<commit_message>
updated the presentation slides
</commit_message>
<xml_diff>
--- a/data/aqi_census.xlsx
+++ b/data/aqi_census.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1323,2154 +1323,2154 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>2020</v>
       </c>
       <c r="D22" t="n">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>19.63</v>
+        <v>1572.46</v>
       </c>
       <c r="H22" t="n">
-        <v>1763000</v>
+        <v>716000</v>
       </c>
       <c r="I22" t="n">
-        <v>89811.50999999999</v>
+        <v>455.34</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Cleveland, MS</t>
+          <t>Columbia, SC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>2021</v>
       </c>
       <c r="D23" t="n">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>19.63</v>
+        <v>1572.46</v>
       </c>
       <c r="H23" t="n">
-        <v>1760000</v>
+        <v>730000</v>
       </c>
       <c r="I23" t="n">
-        <v>89658.69</v>
+        <v>464.24</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Cleveland, MS</t>
+          <t>Columbia, SC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>2022</v>
       </c>
       <c r="D24" t="n">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>19.63</v>
+        <v>1572.46</v>
       </c>
       <c r="H24" t="n">
-        <v>1761000</v>
+        <v>743000</v>
       </c>
       <c r="I24" t="n">
-        <v>89709.63</v>
+        <v>472.51</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Cleveland, MS</t>
+          <t>Columbia, SC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>2023</v>
       </c>
       <c r="D25" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>19.63</v>
+        <v>1572.46</v>
       </c>
       <c r="H25" t="n">
-        <v>1764000</v>
+        <v>755000</v>
       </c>
       <c r="I25" t="n">
-        <v>89862.46000000001</v>
+        <v>480.14</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Cleveland, MS</t>
+          <t>Columbia, SC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>2024</v>
       </c>
       <c r="D26" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Cleveland</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>19.63</v>
+        <v>1572.46</v>
       </c>
       <c r="H26" t="n">
-        <v>1771000</v>
+        <v>766000</v>
       </c>
       <c r="I26" t="n">
-        <v>90219.05</v>
+        <v>487.13</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Cleveland, MS</t>
+          <t>Columbia, SC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>2020</v>
       </c>
       <c r="D27" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1572.46</v>
+        <v>958.12</v>
       </c>
       <c r="H27" t="n">
-        <v>716000</v>
+        <v>384000</v>
       </c>
       <c r="I27" t="n">
-        <v>455.34</v>
+        <v>400.78</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Columbia, SC</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>2021</v>
       </c>
       <c r="D28" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1572.46</v>
+        <v>958.12</v>
       </c>
       <c r="H28" t="n">
-        <v>730000</v>
+        <v>392000</v>
       </c>
       <c r="I28" t="n">
-        <v>464.24</v>
+        <v>409.13</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Columbia, SC</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>2022</v>
       </c>
       <c r="D29" t="n">
-        <v>43</v>
+        <v>74</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1572.46</v>
+        <v>958.12</v>
       </c>
       <c r="H29" t="n">
-        <v>743000</v>
+        <v>400000</v>
       </c>
       <c r="I29" t="n">
-        <v>472.51</v>
+        <v>417.48</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Columbia, SC</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>2023</v>
       </c>
       <c r="D30" t="n">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1572.46</v>
+        <v>958.12</v>
       </c>
       <c r="H30" t="n">
-        <v>755000</v>
+        <v>407000</v>
       </c>
       <c r="I30" t="n">
-        <v>480.14</v>
+        <v>424.79</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Columbia, SC</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>2024</v>
       </c>
       <c r="D31" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Huntsville</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1572.46</v>
+        <v>958.12</v>
       </c>
       <c r="H31" t="n">
-        <v>766000</v>
+        <v>414000</v>
       </c>
       <c r="I31" t="n">
-        <v>487.13</v>
+        <v>432.1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Columbia, SC</t>
+          <t>Huntsville, AL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>2020</v>
       </c>
       <c r="D32" t="n">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>958.12</v>
+        <v>639.64</v>
       </c>
       <c r="H32" t="n">
-        <v>384000</v>
+        <v>420000</v>
       </c>
       <c r="I32" t="n">
-        <v>400.78</v>
+        <v>656.62</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Jackson, MS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>2021</v>
       </c>
       <c r="D33" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>958.12</v>
+        <v>639.64</v>
       </c>
       <c r="H33" t="n">
-        <v>392000</v>
+        <v>426000</v>
       </c>
       <c r="I33" t="n">
-        <v>409.13</v>
+        <v>666</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Jackson, MS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>2022</v>
       </c>
       <c r="D34" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>958.12</v>
+        <v>639.64</v>
       </c>
       <c r="H34" t="n">
-        <v>400000</v>
+        <v>431000</v>
       </c>
       <c r="I34" t="n">
-        <v>417.48</v>
+        <v>673.8200000000001</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Jackson, MS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>2023</v>
       </c>
       <c r="D35" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>958.12</v>
+        <v>639.64</v>
       </c>
       <c r="H35" t="n">
-        <v>407000</v>
+        <v>436000</v>
       </c>
       <c r="I35" t="n">
-        <v>424.79</v>
+        <v>681.63</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Jackson, MS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>2024</v>
       </c>
       <c r="D36" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Huntsville</t>
+          <t>Jackson</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>958.12</v>
+        <v>639.64</v>
       </c>
       <c r="H36" t="n">
-        <v>414000</v>
+        <v>441000</v>
       </c>
       <c r="I36" t="n">
-        <v>432.1</v>
+        <v>689.45</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Huntsville, AL</t>
+          <t>Jackson, MS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>2020</v>
       </c>
       <c r="D37" t="n">
-        <v>22</v>
+        <v>115</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>639.64</v>
+        <v>2703.65</v>
       </c>
       <c r="H37" t="n">
-        <v>420000</v>
+        <v>1686000</v>
       </c>
       <c r="I37" t="n">
-        <v>656.62</v>
+        <v>623.6</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Jackson, MS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>2021</v>
       </c>
       <c r="D38" t="n">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>639.64</v>
+        <v>2703.65</v>
       </c>
       <c r="H38" t="n">
-        <v>426000</v>
+        <v>1698000</v>
       </c>
       <c r="I38" t="n">
-        <v>666</v>
+        <v>628.04</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Jackson, MS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>2022</v>
       </c>
       <c r="D39" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>639.64</v>
+        <v>2703.65</v>
       </c>
       <c r="H39" t="n">
-        <v>431000</v>
+        <v>1711000</v>
       </c>
       <c r="I39" t="n">
-        <v>673.8200000000001</v>
+        <v>632.85</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Jackson, MS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>2023</v>
       </c>
       <c r="D40" t="n">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>639.64</v>
+        <v>2703.65</v>
       </c>
       <c r="H40" t="n">
-        <v>436000</v>
+        <v>1725000</v>
       </c>
       <c r="I40" t="n">
-        <v>681.63</v>
+        <v>638.03</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Jackson, MS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C41" t="n">
         <v>2024</v>
       </c>
       <c r="D41" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Jackson</t>
+          <t>Kansas City</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>639.64</v>
+        <v>2703.65</v>
       </c>
       <c r="H41" t="n">
-        <v>441000</v>
+        <v>1739000</v>
       </c>
       <c r="I41" t="n">
-        <v>689.45</v>
+        <v>643.2</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Jackson, MS</t>
+          <t>Kansas City, MO</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>2020</v>
       </c>
       <c r="D42" t="n">
-        <v>115</v>
+        <v>52</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2703.65</v>
+        <v>816.03</v>
       </c>
       <c r="H42" t="n">
-        <v>1686000</v>
+        <v>741000</v>
       </c>
       <c r="I42" t="n">
-        <v>623.6</v>
+        <v>908.05</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C43" t="n">
         <v>2021</v>
       </c>
       <c r="D43" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>2703.65</v>
+        <v>816.03</v>
       </c>
       <c r="H43" t="n">
-        <v>1698000</v>
+        <v>756000</v>
       </c>
       <c r="I43" t="n">
-        <v>628.04</v>
+        <v>926.4400000000001</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>2022</v>
       </c>
       <c r="D44" t="n">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>2703.65</v>
+        <v>816.03</v>
       </c>
       <c r="H44" t="n">
-        <v>1711000</v>
+        <v>771000</v>
       </c>
       <c r="I44" t="n">
-        <v>632.85</v>
+        <v>944.8200000000001</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>2023</v>
       </c>
       <c r="D45" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>2703.65</v>
+        <v>816.03</v>
       </c>
       <c r="H45" t="n">
-        <v>1725000</v>
+        <v>784000</v>
       </c>
       <c r="I45" t="n">
-        <v>638.03</v>
+        <v>960.75</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>2024</v>
       </c>
       <c r="D46" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Knoxville</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2703.65</v>
+        <v>816.03</v>
       </c>
       <c r="H46" t="n">
-        <v>1739000</v>
+        <v>796000</v>
       </c>
       <c r="I46" t="n">
-        <v>643.2</v>
+        <v>975.45</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Kansas City, MO</t>
+          <t>Knoxville, TN</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C47" t="n">
         <v>2020</v>
       </c>
       <c r="D47" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>816.03</v>
+        <v>724.67</v>
       </c>
       <c r="H47" t="n">
-        <v>741000</v>
+        <v>514000</v>
       </c>
       <c r="I47" t="n">
-        <v>908.05</v>
+        <v>709.29</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Little Rock, AR</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>2021</v>
       </c>
       <c r="D48" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>816.03</v>
+        <v>724.67</v>
       </c>
       <c r="H48" t="n">
-        <v>756000</v>
+        <v>521000</v>
       </c>
       <c r="I48" t="n">
-        <v>926.4400000000001</v>
+        <v>718.95</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Little Rock, AR</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C49" t="n">
         <v>2022</v>
       </c>
       <c r="D49" t="n">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>816.03</v>
+        <v>724.67</v>
       </c>
       <c r="H49" t="n">
-        <v>771000</v>
+        <v>527000</v>
       </c>
       <c r="I49" t="n">
-        <v>944.8200000000001</v>
+        <v>727.23</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Little Rock, AR</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>2023</v>
       </c>
       <c r="D50" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>816.03</v>
+        <v>724.67</v>
       </c>
       <c r="H50" t="n">
-        <v>784000</v>
+        <v>533000</v>
       </c>
       <c r="I50" t="n">
-        <v>960.75</v>
+        <v>735.51</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Little Rock, AR</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>2024</v>
       </c>
       <c r="D51" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Knoxville</t>
+          <t>Little Rock</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="G51" t="n">
-        <v>816.03</v>
+        <v>724.67</v>
       </c>
       <c r="H51" t="n">
-        <v>796000</v>
+        <v>539000</v>
       </c>
       <c r="I51" t="n">
-        <v>975.45</v>
+        <v>743.79</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Knoxville, TN</t>
+          <t>Little Rock, AR</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>2020</v>
       </c>
       <c r="D52" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="G52" t="n">
-        <v>724.67</v>
+        <v>1048.12</v>
       </c>
       <c r="H52" t="n">
-        <v>514000</v>
+        <v>1089000</v>
       </c>
       <c r="I52" t="n">
-        <v>709.29</v>
+        <v>1039</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Little Rock, AR</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>2021</v>
       </c>
       <c r="D53" t="n">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="G53" t="n">
-        <v>724.67</v>
+        <v>1048.12</v>
       </c>
       <c r="H53" t="n">
-        <v>521000</v>
+        <v>1098000</v>
       </c>
       <c r="I53" t="n">
-        <v>718.95</v>
+        <v>1047.59</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Little Rock, AR</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>2022</v>
       </c>
       <c r="D54" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="G54" t="n">
-        <v>724.67</v>
+        <v>1048.12</v>
       </c>
       <c r="H54" t="n">
-        <v>527000</v>
+        <v>1107000</v>
       </c>
       <c r="I54" t="n">
-        <v>727.23</v>
+        <v>1056.18</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Little Rock, AR</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="C55" t="n">
         <v>2023</v>
       </c>
       <c r="D55" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="G55" t="n">
-        <v>724.67</v>
+        <v>1048.12</v>
       </c>
       <c r="H55" t="n">
-        <v>533000</v>
+        <v>1116000</v>
       </c>
       <c r="I55" t="n">
-        <v>735.51</v>
+        <v>1064.76</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Little Rock, AR</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>2024</v>
       </c>
       <c r="D56" t="n">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Little Rock</t>
+          <t>Louisville</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="G56" t="n">
-        <v>724.67</v>
+        <v>1048.12</v>
       </c>
       <c r="H56" t="n">
-        <v>539000</v>
+        <v>1126000</v>
       </c>
       <c r="I56" t="n">
-        <v>743.79</v>
+        <v>1074.3</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Little Rock, AR</t>
+          <t>Louisville, KY</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>2020</v>
       </c>
       <c r="D57" t="n">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G57" t="n">
-        <v>1048.12</v>
+        <v>1232.87</v>
       </c>
       <c r="H57" t="n">
-        <v>1089000</v>
+        <v>1150000</v>
       </c>
       <c r="I57" t="n">
-        <v>1039</v>
+        <v>932.78</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>2021</v>
       </c>
       <c r="D58" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G58" t="n">
-        <v>1048.12</v>
+        <v>1232.87</v>
       </c>
       <c r="H58" t="n">
-        <v>1098000</v>
+        <v>1156000</v>
       </c>
       <c r="I58" t="n">
-        <v>1047.59</v>
+        <v>937.65</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>2022</v>
       </c>
       <c r="D59" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1048.12</v>
+        <v>1232.87</v>
       </c>
       <c r="H59" t="n">
-        <v>1107000</v>
+        <v>1163000</v>
       </c>
       <c r="I59" t="n">
-        <v>1056.18</v>
+        <v>943.33</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C60" t="n">
         <v>2023</v>
       </c>
       <c r="D60" t="n">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G60" t="n">
-        <v>1048.12</v>
+        <v>1232.87</v>
       </c>
       <c r="H60" t="n">
-        <v>1116000</v>
+        <v>1170000</v>
       </c>
       <c r="I60" t="n">
-        <v>1064.76</v>
+        <v>949.01</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>2024</v>
       </c>
       <c r="D61" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Louisville</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>KY</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G61" t="n">
-        <v>1048.12</v>
+        <v>1232.87</v>
       </c>
       <c r="H61" t="n">
-        <v>1126000</v>
+        <v>1179000</v>
       </c>
       <c r="I61" t="n">
-        <v>1074.3</v>
+        <v>956.3099999999999</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Louisville, KY</t>
+          <t>Memphis, TN</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>2020</v>
       </c>
       <c r="D62" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G62" t="n">
-        <v>1232.87</v>
+        <v>683.97</v>
       </c>
       <c r="H62" t="n">
-        <v>1150000</v>
+        <v>333000</v>
       </c>
       <c r="I62" t="n">
-        <v>932.78</v>
+        <v>486.86</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mobile, AL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>2021</v>
       </c>
       <c r="D63" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1232.87</v>
+        <v>683.97</v>
       </c>
       <c r="H63" t="n">
-        <v>1156000</v>
+        <v>333000</v>
       </c>
       <c r="I63" t="n">
-        <v>937.65</v>
+        <v>486.86</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mobile, AL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>2022</v>
       </c>
       <c r="D64" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>1232.87</v>
+        <v>683.97</v>
       </c>
       <c r="H64" t="n">
-        <v>1163000</v>
+        <v>334000</v>
       </c>
       <c r="I64" t="n">
-        <v>943.33</v>
+        <v>488.33</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mobile, AL</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>2023</v>
       </c>
       <c r="D65" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1232.87</v>
+        <v>683.97</v>
       </c>
       <c r="H65" t="n">
-        <v>1170000</v>
+        <v>335000</v>
       </c>
       <c r="I65" t="n">
-        <v>949.01</v>
+        <v>489.79</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mobile, AL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>2024</v>
       </c>
       <c r="D66" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1232.87</v>
+        <v>683.97</v>
       </c>
       <c r="H66" t="n">
-        <v>1179000</v>
+        <v>337000</v>
       </c>
       <c r="I66" t="n">
-        <v>956.3099999999999</v>
+        <v>492.71</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Memphis, TN</t>
+          <t>Mobile, AL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C67" t="n">
         <v>2020</v>
       </c>
       <c r="D67" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G67" t="n">
-        <v>683.97</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="H67" t="n">
-        <v>333000</v>
+        <v>377000</v>
       </c>
       <c r="I67" t="n">
-        <v>486.86</v>
+        <v>710.0700000000001</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Mobile, AL</t>
+          <t>Myrtle Beach, SC</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C68" t="n">
         <v>2021</v>
       </c>
       <c r="D68" t="n">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G68" t="n">
-        <v>683.97</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="H68" t="n">
-        <v>333000</v>
+        <v>393000</v>
       </c>
       <c r="I68" t="n">
-        <v>486.86</v>
+        <v>740.21</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Mobile, AL</t>
+          <t>Myrtle Beach, SC</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C69" t="n">
         <v>2022</v>
       </c>
       <c r="D69" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G69" t="n">
-        <v>683.97</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="H69" t="n">
-        <v>334000</v>
+        <v>408000</v>
       </c>
       <c r="I69" t="n">
-        <v>488.33</v>
+        <v>768.46</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Mobile, AL</t>
+          <t>Myrtle Beach, SC</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C70" t="n">
         <v>2023</v>
       </c>
       <c r="D70" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G70" t="n">
-        <v>683.97</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="H70" t="n">
-        <v>335000</v>
+        <v>421000</v>
       </c>
       <c r="I70" t="n">
-        <v>489.79</v>
+        <v>792.95</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Mobile, AL</t>
+          <t>Myrtle Beach, SC</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="C71" t="n">
         <v>2024</v>
       </c>
       <c r="D71" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Myrtle Beach</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>683.97</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="H71" t="n">
-        <v>337000</v>
+        <v>432000</v>
       </c>
       <c r="I71" t="n">
-        <v>492.71</v>
+        <v>813.67</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Mobile, AL</t>
+          <t>Myrtle Beach, SC</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>2020</v>
       </c>
       <c r="D72" t="n">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G72" t="n">
-        <v>530.9299999999999</v>
+        <v>2121.45</v>
       </c>
       <c r="H72" t="n">
-        <v>377000</v>
+        <v>1249000</v>
       </c>
       <c r="I72" t="n">
-        <v>710.0700000000001</v>
+        <v>588.75</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Myrtle Beach, SC</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -3481,206 +3481,206 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>530.9299999999999</v>
+        <v>2121.45</v>
       </c>
       <c r="H73" t="n">
-        <v>393000</v>
+        <v>1272000</v>
       </c>
       <c r="I73" t="n">
-        <v>740.21</v>
+        <v>599.59</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Myrtle Beach, SC</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>2022</v>
       </c>
       <c r="D74" t="n">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G74" t="n">
-        <v>530.9299999999999</v>
+        <v>2121.45</v>
       </c>
       <c r="H74" t="n">
-        <v>408000</v>
+        <v>1294000</v>
       </c>
       <c r="I74" t="n">
-        <v>768.46</v>
+        <v>609.96</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Myrtle Beach, SC</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C75" t="n">
         <v>2023</v>
       </c>
       <c r="D75" t="n">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G75" t="n">
-        <v>530.9299999999999</v>
+        <v>2121.45</v>
       </c>
       <c r="H75" t="n">
-        <v>421000</v>
+        <v>1315000</v>
       </c>
       <c r="I75" t="n">
-        <v>792.95</v>
+        <v>619.86</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Myrtle Beach, SC</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="C76" t="n">
         <v>2024</v>
       </c>
       <c r="D76" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Myrtle Beach</t>
+          <t>Nashville</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>TN</t>
         </is>
       </c>
       <c r="G76" t="n">
-        <v>530.9299999999999</v>
+        <v>2121.45</v>
       </c>
       <c r="H76" t="n">
-        <v>432000</v>
+        <v>1333000</v>
       </c>
       <c r="I76" t="n">
-        <v>813.67</v>
+        <v>628.34</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Myrtle Beach, SC</t>
+          <t>Nashville, TN</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>2020</v>
       </c>
       <c r="D77" t="n">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="G77" t="n">
-        <v>2121.45</v>
+        <v>737.35</v>
       </c>
       <c r="H77" t="n">
-        <v>1249000</v>
+        <v>1105000</v>
       </c>
       <c r="I77" t="n">
-        <v>588.75</v>
+        <v>1498.61</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -3691,164 +3691,164 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="G78" t="n">
-        <v>2121.45</v>
+        <v>737.35</v>
       </c>
       <c r="H78" t="n">
-        <v>1272000</v>
+        <v>1117000</v>
       </c>
       <c r="I78" t="n">
-        <v>599.59</v>
+        <v>1514.88</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="C79" t="n">
         <v>2022</v>
       </c>
       <c r="D79" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="G79" t="n">
-        <v>2121.45</v>
+        <v>737.35</v>
       </c>
       <c r="H79" t="n">
-        <v>1294000</v>
+        <v>1128000</v>
       </c>
       <c r="I79" t="n">
-        <v>609.96</v>
+        <v>1529.8</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="C80" t="n">
         <v>2023</v>
       </c>
       <c r="D80" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="G80" t="n">
-        <v>2121.45</v>
+        <v>737.35</v>
       </c>
       <c r="H80" t="n">
-        <v>1315000</v>
+        <v>1140000</v>
       </c>
       <c r="I80" t="n">
-        <v>619.86</v>
+        <v>1546.08</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="C81" t="n">
         <v>2024</v>
       </c>
       <c r="D81" t="n">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Nashville</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>TN</t>
+          <t>VA</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>2121.45</v>
+        <v>737.35</v>
       </c>
       <c r="H81" t="n">
-        <v>1333000</v>
+        <v>1151000</v>
       </c>
       <c r="I81" t="n">
-        <v>628.34</v>
+        <v>1561</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Nashville, TN</t>
+          <t>Richmond, VA</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -3859,80 +3859,80 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>737.35</v>
+        <v>607.97</v>
       </c>
       <c r="H82" t="n">
-        <v>1105000</v>
+        <v>324000</v>
       </c>
       <c r="I82" t="n">
-        <v>1498.61</v>
+        <v>532.92</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C83" t="n">
         <v>2021</v>
       </c>
       <c r="D83" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>737.35</v>
+        <v>607.97</v>
       </c>
       <c r="H83" t="n">
-        <v>1117000</v>
+        <v>329000</v>
       </c>
       <c r="I83" t="n">
-        <v>1514.88</v>
+        <v>541.15</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -3943,122 +3943,122 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="G84" t="n">
-        <v>737.35</v>
+        <v>607.97</v>
       </c>
       <c r="H84" t="n">
-        <v>1128000</v>
+        <v>334000</v>
       </c>
       <c r="I84" t="n">
-        <v>1529.8</v>
+        <v>549.37</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C85" t="n">
         <v>2023</v>
       </c>
       <c r="D85" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="G85" t="n">
-        <v>737.35</v>
+        <v>607.97</v>
       </c>
       <c r="H85" t="n">
-        <v>1140000</v>
+        <v>339000</v>
       </c>
       <c r="I85" t="n">
-        <v>1546.08</v>
+        <v>557.59</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="C86" t="n">
         <v>2024</v>
       </c>
       <c r="D86" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Richmond</t>
+          <t>Savannah</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>VA</t>
+          <t>GA</t>
         </is>
       </c>
       <c r="G86" t="n">
-        <v>737.35</v>
+        <v>607.97</v>
       </c>
       <c r="H86" t="n">
-        <v>1151000</v>
+        <v>343000</v>
       </c>
       <c r="I86" t="n">
-        <v>1561</v>
+        <v>564.17</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Richmond, VA</t>
+          <t>Savannah, GA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -4069,80 +4069,80 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>607.97</v>
+        <v>368.02</v>
       </c>
       <c r="H87" t="n">
-        <v>324000</v>
+        <v>669000</v>
       </c>
       <c r="I87" t="n">
-        <v>532.92</v>
+        <v>1817.84</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Savannah, GA</t>
+          <t>Springfield, MO</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>2021</v>
       </c>
       <c r="D88" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G88" t="n">
-        <v>607.97</v>
+        <v>368.02</v>
       </c>
       <c r="H88" t="n">
-        <v>329000</v>
+        <v>672000</v>
       </c>
       <c r="I88" t="n">
-        <v>541.15</v>
+        <v>1825.99</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Savannah, GA</t>
+          <t>Springfield, MO</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -4153,318 +4153,108 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>607.97</v>
+        <v>368.02</v>
       </c>
       <c r="H89" t="n">
-        <v>334000</v>
+        <v>676000</v>
       </c>
       <c r="I89" t="n">
-        <v>549.37</v>
+        <v>1836.86</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Savannah, GA</t>
+          <t>Springfield, MO</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C90" t="n">
         <v>2023</v>
       </c>
       <c r="D90" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G90" t="n">
-        <v>607.97</v>
+        <v>368.02</v>
       </c>
       <c r="H90" t="n">
-        <v>339000</v>
+        <v>680000</v>
       </c>
       <c r="I90" t="n">
-        <v>557.59</v>
+        <v>1847.73</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Savannah, GA</t>
+          <t>Springfield, MO</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C91" t="n">
         <v>2024</v>
       </c>
       <c r="D91" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Savannah</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>GA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="G91" t="n">
-        <v>607.97</v>
+        <v>368.02</v>
       </c>
       <c r="H91" t="n">
-        <v>343000</v>
+        <v>685000</v>
       </c>
       <c r="I91" t="n">
-        <v>564.17</v>
+        <v>1861.31</v>
       </c>
       <c r="J91" t="inlineStr">
-        <is>
-          <t>Savannah, GA</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="C92" t="n">
-        <v>2020</v>
-      </c>
-      <c r="D92" t="n">
-        <v>35</v>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G92" t="n">
-        <v>368.02</v>
-      </c>
-      <c r="H92" t="n">
-        <v>669000</v>
-      </c>
-      <c r="I92" t="n">
-        <v>1817.84</v>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>Springfield, MO</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="C93" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D93" t="n">
-        <v>35</v>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G93" t="n">
-        <v>368.02</v>
-      </c>
-      <c r="H93" t="n">
-        <v>672000</v>
-      </c>
-      <c r="I93" t="n">
-        <v>1825.99</v>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>Springfield, MO</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D94" t="n">
-        <v>35</v>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G94" t="n">
-        <v>368.02</v>
-      </c>
-      <c r="H94" t="n">
-        <v>676000</v>
-      </c>
-      <c r="I94" t="n">
-        <v>1836.86</v>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Springfield, MO</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D95" t="n">
-        <v>40</v>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G95" t="n">
-        <v>368.02</v>
-      </c>
-      <c r="H95" t="n">
-        <v>680000</v>
-      </c>
-      <c r="I95" t="n">
-        <v>1847.73</v>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>Springfield, MO</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D96" t="n">
-        <v>26</v>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>Springfield</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>MO</t>
-        </is>
-      </c>
-      <c r="G96" t="n">
-        <v>368.02</v>
-      </c>
-      <c r="H96" t="n">
-        <v>685000</v>
-      </c>
-      <c r="I96" t="n">
-        <v>1861.31</v>
-      </c>
-      <c r="J96" t="inlineStr">
         <is>
           <t>Springfield, MO</t>
         </is>

</xml_diff>